<commit_message>
feat(phase1-0B): VSME/ESG/Finance services, models, routers + CC_* named ranges
- Add CC_* named ranges (49 ESG, 28 Finance) + _Manifest sheet to all 3 workbooks
- models/vsme.py: VSME snapshot (profile, environnement, social, gouvernance, complétude)
- models/esg.py: ESG snapshot (matérialité IRO, scores E/S/G, QC controls)
- models/finance.py: Finance snapshot (finance climat, SFDR PAI 14, benchmark sectoriel)
- services/esg_service.py: build_vsme_snapshot() + build_esg_snapshot() with CC_* fallbacks
- services/finance_service.py: build_finance_snapshot() with benchmark sector reference data
- routers/vsme.py: GET /vsme/snapshot
- routers/esg.py: GET /esg/snapshot
- routers/finance.py: GET /finance/snapshot
- main.py: register vsme, esg, finance routers

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/apps/api/data/CarbonCo_Calcul_Carbone_v2.xlsx
+++ b/apps/api/data/CarbonCo_Calcul_Carbone_v2.xlsx
@@ -46,6 +46,7 @@
     <sheet name="12_USAGES_NUMÉRIQUES" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="13_MODÉLISATION_SERVICES" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="14_SYNTHÈSE_GLOBALE" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="_Manifest" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames>
     <definedName name="Annee_Reporting">"Paramètres!$B$7"</definedName>
@@ -15672,9 +15673,9 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="A12:J12"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A12:J12"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="C14:C23 E14:F23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Erreur de saisie" error="Valeur non autorisée" type="list">
@@ -54815,6 +54816,87 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>CarbonCo_Calcul_Carbone_v2 — Manifest</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Onglets obligatoires</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Couverture,Sommaire,Parametres,Synthese_GES,Energie,Trajectoire_SBTi,CBAM,Taxonomie,_Controles_Qualite,Claude Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Plages CC_* requises</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Controles QC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>cf. _Controles_Qualite</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>